<commit_message>
Business case v11: snapshot before untracking (last version kept in history)
</commit_message>
<xml_diff>
--- a/assets/Aevia - Business case v11.xlsx
+++ b/assets/Aevia - Business case v11.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\evgmy\aevia-test\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98330364-CE45-4B40-A2B0-BFCE928C6EDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65CF6A1C-2D42-41A5-BE63-5D91062865A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Periodika" sheetId="1" state="hidden" r:id="rId1"/>
@@ -3203,7 +3203,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="188">
+  <cellXfs count="186">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3463,13 +3463,11 @@
     <xf numFmtId="3" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -11331,40 +11329,40 @@
       <c r="E21" t="s">
         <v>33</v>
       </c>
-      <c r="G21" s="187">
-        <v>0</v>
-      </c>
-      <c r="H21" s="187">
-        <v>0</v>
-      </c>
-      <c r="I21" s="187">
+      <c r="G21" s="183">
+        <v>0</v>
+      </c>
+      <c r="H21" s="183">
+        <v>0</v>
+      </c>
+      <c r="I21" s="183">
         <v>5</v>
       </c>
-      <c r="J21" s="187">
+      <c r="J21" s="183">
         <v>10</v>
       </c>
-      <c r="K21" s="187">
+      <c r="K21" s="183">
         <v>20</v>
       </c>
-      <c r="L21" s="187">
+      <c r="L21" s="183">
         <v>30</v>
       </c>
-      <c r="M21" s="187">
+      <c r="M21" s="183">
         <v>40</v>
       </c>
-      <c r="N21" s="187">
+      <c r="N21" s="183">
         <v>50</v>
       </c>
-      <c r="O21" s="187">
+      <c r="O21" s="183">
         <v>65</v>
       </c>
-      <c r="P21" s="187">
+      <c r="P21" s="183">
         <v>80</v>
       </c>
-      <c r="Q21" s="187">
+      <c r="Q21" s="183">
         <v>95</v>
       </c>
-      <c r="R21" s="187">
+      <c r="R21" s="183">
         <v>110</v>
       </c>
       <c r="T21" t="s">
@@ -11856,27 +11854,27 @@
       <c r="L34" s="175">
         <v>0</v>
       </c>
-      <c r="M34" s="185">
+      <c r="M34" s="175">
         <f t="shared" ref="M34:R34" si="11">$F$54*I31</f>
         <v>1</v>
       </c>
-      <c r="N34" s="185">
+      <c r="N34" s="175">
         <f t="shared" si="11"/>
         <v>9.2783505154639183</v>
       </c>
-      <c r="O34" s="185">
+      <c r="O34" s="175">
         <f t="shared" si="11"/>
         <v>16.458333333333336</v>
       </c>
-      <c r="P34" s="185">
+      <c r="P34" s="175">
         <f t="shared" si="11"/>
         <v>23.333333333333336</v>
       </c>
-      <c r="Q34" s="185">
+      <c r="Q34" s="175">
         <f t="shared" si="11"/>
         <v>30.736842105263165</v>
       </c>
-      <c r="R34" s="185">
+      <c r="R34" s="175">
         <f t="shared" si="11"/>
         <v>37.684210526315795</v>
       </c>
@@ -12525,7 +12523,7 @@
       <c r="D54" t="s">
         <v>75</v>
       </c>
-      <c r="F54" s="186">
+      <c r="F54">
         <v>0.2</v>
       </c>
       <c r="T54" t="s">
@@ -16219,16 +16217,16 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="E3" s="183" t="s">
+      <c r="E3" s="184" t="s">
         <v>380</v>
       </c>
-      <c r="F3" s="184"/>
-      <c r="G3" s="184"/>
-      <c r="H3" s="183" t="s">
+      <c r="F3" s="185"/>
+      <c r="G3" s="185"/>
+      <c r="H3" s="184" t="s">
         <v>381</v>
       </c>
-      <c r="I3" s="184"/>
-      <c r="J3" s="184"/>
+      <c r="I3" s="185"/>
+      <c r="J3" s="185"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B4" t="s">

</xml_diff>